<commit_message>
fixes to timesheet imports from replicon
</commit_message>
<xml_diff>
--- a/uploads/replicon_mapping.xlsx
+++ b/uploads/replicon_mapping.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joshu\Documents\Repos\ReadyGo\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{88B6387F-02BA-4DD7-931B-608ED835640C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{884DF782-1CA6-4587-9D68-F5F8C472021B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{4C2A3FAA-68E7-4292-8E90-23EC27F02F7D}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4C2A3FAA-68E7-4292-8E90-23EC27F02F7D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="591" uniqueCount="252">
   <si>
     <t>Accelerant - WS Audiology</t>
   </si>
@@ -820,6 +819,24 @@
   </si>
   <si>
     <t>Engagement - Lilly Pulitzer - ERP Implementation (staff aug)</t>
+  </si>
+  <si>
+    <t>PH Training - Arch</t>
+  </si>
+  <si>
+    <t>AU PTO - Arch</t>
+  </si>
+  <si>
+    <t>US PTO - Arch</t>
+  </si>
+  <si>
+    <t>US Training - Ach</t>
+  </si>
+  <si>
+    <t>US Bench _ Arch</t>
+  </si>
+  <si>
+    <t>US Bench</t>
   </si>
 </sst>
 </file>
@@ -873,7 +890,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -894,10 +911,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1234,7 +1247,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C21748B-2ADD-42E6-BB3D-0F02ECC523B7}">
-  <dimension ref="A1:G95"/>
+  <dimension ref="A1:G101"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="74.5546875" bestFit="1" customWidth="1"/>
@@ -1269,7 +1282,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="10" t="s">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1290,7 +1303,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1311,7 +1324,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1332,7 +1345,7 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="A5" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1353,7 +1366,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" t="s">
         <v>7</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1377,7 +1390,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="10" t="s">
+      <c r="A7" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1401,7 +1414,7 @@
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="10" t="s">
+      <c r="A8" t="s">
         <v>10</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -1425,7 +1438,7 @@
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="10" t="s">
+      <c r="A9" t="s">
         <v>11</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1449,7 +1462,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
+      <c r="A10" t="s">
         <v>12</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -1473,7 +1486,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
+      <c r="A11" t="s">
         <v>13</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1497,7 +1510,7 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="10" t="s">
+      <c r="A12" t="s">
         <v>14</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1521,7 +1534,7 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="10" t="s">
+      <c r="A13" t="s">
         <v>15</v>
       </c>
       <c r="B13" t="s">
@@ -1540,7 +1553,7 @@
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="10" t="s">
+      <c r="A14" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1564,7 +1577,7 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="10" t="s">
+      <c r="A15" t="s">
         <v>17</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1583,7 +1596,7 @@
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="10" t="s">
+      <c r="A16" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1602,7 +1615,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" s="10" t="s">
+      <c r="A17" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1621,11 +1634,11 @@
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
+      <c r="A18" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="C18" s="2" t="s">
         <v>239</v>
@@ -1640,7 +1653,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="10" t="s">
+      <c r="A19" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1660,7 +1673,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="10" t="s">
+      <c r="A20" t="s">
         <v>24</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1680,7 +1693,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="10" t="s">
+      <c r="A21" t="s">
         <v>25</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1699,7 +1712,7 @@
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" s="10" t="s">
+      <c r="A22" t="s">
         <v>26</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1718,7 +1731,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" s="10" t="s">
+      <c r="A23" t="s">
         <v>27</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1737,7 +1750,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" s="10" t="s">
+      <c r="A24" t="s">
         <v>28</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1757,7 +1770,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" s="10" t="s">
+      <c r="A25" t="s">
         <v>29</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -1776,7 +1789,7 @@
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" s="10" t="s">
+      <c r="A26" t="s">
         <v>30</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -1795,7 +1808,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A27" s="10" t="s">
+      <c r="A27" t="s">
         <v>32</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -1815,7 +1828,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A28" s="10" t="s">
+      <c r="A28" t="s">
         <v>33</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -1834,7 +1847,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A29" s="10" t="s">
+      <c r="A29" t="s">
         <v>34</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -1854,7 +1867,7 @@
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A30" s="10" t="s">
+      <c r="A30" t="s">
         <v>36</v>
       </c>
       <c r="B30" s="1" t="s">
@@ -1874,7 +1887,7 @@
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A31" s="10" t="s">
+      <c r="A31" t="s">
         <v>38</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -1894,7 +1907,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A32" s="10" t="s">
+      <c r="A32" t="s">
         <v>39</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -1914,7 +1927,7 @@
       </c>
     </row>
     <row r="33" spans="1:7" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A33" s="10" t="s">
+      <c r="A33" t="s">
         <v>41</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -1935,7 +1948,7 @@
       </c>
     </row>
     <row r="34" spans="1:7" ht="216" x14ac:dyDescent="0.3">
-      <c r="A34" s="10" t="s">
+      <c r="A34" t="s">
         <v>43</v>
       </c>
       <c r="B34" s="1" t="s">
@@ -1956,7 +1969,7 @@
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="10" t="s">
+      <c r="A35" t="s">
         <v>44</v>
       </c>
       <c r="B35" s="1" t="s">
@@ -1975,7 +1988,7 @@
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
+      <c r="A36" t="s">
         <v>46</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -1995,7 +2008,7 @@
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="10" t="s">
+      <c r="A37" t="s">
         <v>48</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -2015,7 +2028,7 @@
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="10" t="s">
+      <c r="A38" t="s">
         <v>50</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -2035,7 +2048,7 @@
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="10" t="s">
+      <c r="A39" t="s">
         <v>51</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -2052,7 +2065,7 @@
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="10" t="s">
+      <c r="A40" t="s">
         <v>52</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -2072,7 +2085,7 @@
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A41" s="10" t="s">
+      <c r="A41" t="s">
         <v>54</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -2092,7 +2105,7 @@
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A42" s="10" t="s">
+      <c r="A42" t="s">
         <v>56</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -2112,7 +2125,7 @@
       </c>
     </row>
     <row r="43" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A43" s="10" t="s">
+      <c r="A43" t="s">
         <v>57</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -2133,7 +2146,7 @@
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="10" t="s">
+      <c r="A44" t="s">
         <v>59</v>
       </c>
       <c r="B44" s="1" t="s">
@@ -2153,7 +2166,7 @@
       </c>
     </row>
     <row r="45" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="10" t="s">
+      <c r="A45" t="s">
         <v>60</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -2174,7 +2187,7 @@
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="10" t="s">
+      <c r="A46" t="s">
         <v>61</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -2194,7 +2207,7 @@
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="10" t="s">
+      <c r="A47" t="s">
         <v>62</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -2214,7 +2227,7 @@
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="10" t="s">
+      <c r="A48" t="s">
         <v>63</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -2233,7 +2246,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="10" t="s">
+      <c r="A49" t="s">
         <v>65</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -2257,7 +2270,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A50" s="10" t="s">
+      <c r="A50" t="s">
         <v>66</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -2277,7 +2290,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A51" s="10" t="s">
+      <c r="A51" t="s">
         <v>69</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -2286,10 +2299,9 @@
       <c r="C51" t="s">
         <v>182</v>
       </c>
-      <c r="D51" s="10" t="s">
+      <c r="D51" t="s">
         <v>245</v>
       </c>
-      <c r="E51" s="10"/>
       <c r="F51" t="s">
         <v>68</v>
       </c>
@@ -2298,7 +2310,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A52" s="10" t="s">
+      <c r="A52" t="s">
         <v>70</v>
       </c>
       <c r="B52" s="1" t="s">
@@ -2318,7 +2330,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A53" s="10" t="s">
+      <c r="A53" t="s">
         <v>71</v>
       </c>
       <c r="B53" s="1" t="s">
@@ -2339,7 +2351,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A54" s="10" t="s">
+      <c r="A54" t="s">
         <v>73</v>
       </c>
       <c r="B54" s="1" t="s">
@@ -2359,7 +2371,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A55" s="10" t="s">
+      <c r="A55" t="s">
         <v>74</v>
       </c>
       <c r="B55" s="1" t="s">
@@ -2379,7 +2391,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A56" s="10" t="s">
+      <c r="A56" t="s">
         <v>75</v>
       </c>
       <c r="B56" s="1" t="s">
@@ -2399,7 +2411,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="10" t="s">
+      <c r="A57" t="s">
         <v>77</v>
       </c>
       <c r="B57" s="1" t="s">
@@ -2419,7 +2431,7 @@
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A58" s="10" t="s">
+      <c r="A58" t="s">
         <v>79</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -2439,7 +2451,7 @@
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A59" s="10" t="s">
+      <c r="A59" t="s">
         <v>81</v>
       </c>
       <c r="B59" s="1" t="s">
@@ -2459,7 +2471,7 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="10" t="s">
+      <c r="A60" t="s">
         <v>82</v>
       </c>
       <c r="B60" s="1" t="s">
@@ -2479,7 +2491,7 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="10" t="s">
+      <c r="A61" t="s">
         <v>83</v>
       </c>
       <c r="B61" s="1" t="s">
@@ -2499,7 +2511,7 @@
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62" s="10" t="s">
+      <c r="A62" t="s">
         <v>84</v>
       </c>
       <c r="B62" s="1" t="s">
@@ -2523,7 +2535,7 @@
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A63" s="10" t="s">
+      <c r="A63" t="s">
         <v>85</v>
       </c>
       <c r="B63" s="1" t="s">
@@ -2547,7 +2559,7 @@
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A64" s="10" t="s">
+      <c r="A64" t="s">
         <v>86</v>
       </c>
       <c r="B64" s="1" t="s">
@@ -2571,7 +2583,7 @@
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A65" s="10" t="s">
+      <c r="A65" t="s">
         <v>87</v>
       </c>
       <c r="B65" s="1" t="s">
@@ -2595,7 +2607,7 @@
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A66" s="10" t="s">
+      <c r="A66" t="s">
         <v>88</v>
       </c>
       <c r="B66" s="1" t="s">
@@ -2619,7 +2631,7 @@
       </c>
     </row>
     <row r="67" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A67" s="10" t="s">
+      <c r="A67" t="s">
         <v>89</v>
       </c>
       <c r="B67" s="1" t="s">
@@ -2643,7 +2655,7 @@
       </c>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A68" s="10" t="s">
+      <c r="A68" t="s">
         <v>90</v>
       </c>
       <c r="B68" s="1" t="s">
@@ -2656,7 +2668,7 @@
         <f t="shared" si="2"/>
         <v>Engagement - Philippines</v>
       </c>
-      <c r="E68" s="11" t="s">
+      <c r="E68" s="2" t="s">
         <v>230</v>
       </c>
       <c r="F68" t="s">
@@ -2667,7 +2679,7 @@
       </c>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A69" s="10" t="s">
+      <c r="A69" t="s">
         <v>91</v>
       </c>
       <c r="B69" s="1" t="s">
@@ -2691,7 +2703,7 @@
       </c>
     </row>
     <row r="70" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A70" s="10" t="s">
+      <c r="A70" t="s">
         <v>92</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -2715,7 +2727,7 @@
       </c>
     </row>
     <row r="71" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A71" s="10" t="s">
+      <c r="A71" t="s">
         <v>93</v>
       </c>
       <c r="B71" s="1" t="s">
@@ -2736,7 +2748,7 @@
       </c>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A72" s="10" t="s">
+      <c r="A72" t="s">
         <v>94</v>
       </c>
       <c r="B72" s="1" t="s">
@@ -2756,7 +2768,7 @@
       </c>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A73" s="10" t="s">
+      <c r="A73" t="s">
         <v>95</v>
       </c>
       <c r="B73" s="1" t="s">
@@ -2776,7 +2788,7 @@
       </c>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A74" s="10" t="s">
+      <c r="A74" t="s">
         <v>96</v>
       </c>
       <c r="B74" s="1" t="s">
@@ -2796,7 +2808,7 @@
       </c>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A75" s="10" t="s">
+      <c r="A75" t="s">
         <v>97</v>
       </c>
       <c r="B75" s="1" t="s">
@@ -2805,11 +2817,11 @@
       <c r="C75" t="s">
         <v>242</v>
       </c>
-      <c r="D75" s="11" t="s">
+      <c r="D75" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="E75" s="11"/>
-      <c r="F75" s="10" t="s">
+      <c r="E75" s="2"/>
+      <c r="F75" t="s">
         <v>244</v>
       </c>
       <c r="G75" t="s">
@@ -2817,7 +2829,7 @@
       </c>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A76" s="10" t="s">
+      <c r="A76" t="s">
         <v>99</v>
       </c>
       <c r="B76" s="1" t="s">
@@ -2837,7 +2849,7 @@
       </c>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A77" s="10" t="s">
+      <c r="A77" t="s">
         <v>101</v>
       </c>
       <c r="B77" s="1" t="s">
@@ -2857,7 +2869,7 @@
       </c>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A78" s="10" t="s">
+      <c r="A78" t="s">
         <v>102</v>
       </c>
       <c r="B78" s="1" t="s">
@@ -2877,7 +2889,7 @@
       </c>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A79" s="10" t="s">
+      <c r="A79" t="s">
         <v>103</v>
       </c>
       <c r="B79" s="1" t="s">
@@ -2897,7 +2909,7 @@
       </c>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A80" s="10" t="s">
+      <c r="A80" t="s">
         <v>104</v>
       </c>
       <c r="B80" s="1" t="s">
@@ -2917,7 +2929,7 @@
       </c>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A81" s="10" t="s">
+      <c r="A81" t="s">
         <v>105</v>
       </c>
       <c r="B81" s="1" t="s">
@@ -2941,7 +2953,7 @@
       </c>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A82" s="10" t="s">
+      <c r="A82" t="s">
         <v>106</v>
       </c>
       <c r="B82" s="1" t="s">
@@ -2965,7 +2977,7 @@
       </c>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A83" s="10" t="s">
+      <c r="A83" t="s">
         <v>107</v>
       </c>
       <c r="B83" s="1" t="s">
@@ -2989,7 +3001,7 @@
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A84" s="10" t="s">
+      <c r="A84" t="s">
         <v>108</v>
       </c>
       <c r="B84" s="1" t="s">
@@ -3013,7 +3025,7 @@
       </c>
     </row>
     <row r="85" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A85" s="10" t="s">
+      <c r="A85" t="s">
         <v>109</v>
       </c>
       <c r="B85" s="1" t="s">
@@ -3037,7 +3049,7 @@
       </c>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A86" s="10" t="s">
+      <c r="A86" t="s">
         <v>110</v>
       </c>
       <c r="B86" s="1" t="s">
@@ -3061,7 +3073,7 @@
       </c>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A87" s="10" t="s">
+      <c r="A87" t="s">
         <v>111</v>
       </c>
       <c r="B87" s="1" t="s">
@@ -3085,7 +3097,7 @@
       </c>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A88" s="10" t="s">
+      <c r="A88" t="s">
         <v>112</v>
       </c>
       <c r="B88" s="1" t="s">
@@ -3109,7 +3121,7 @@
       </c>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A89" s="10" t="s">
+      <c r="A89" t="s">
         <v>113</v>
       </c>
       <c r="B89" s="1" t="s">
@@ -3128,7 +3140,7 @@
       </c>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A90" s="10" t="s">
+      <c r="A90" t="s">
         <v>115</v>
       </c>
       <c r="B90" s="1" t="s">
@@ -3152,7 +3164,7 @@
       </c>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A91" s="10" t="s">
+      <c r="A91" t="s">
         <v>116</v>
       </c>
       <c r="B91" s="1" t="s">
@@ -3176,7 +3188,7 @@
       </c>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A92" s="10" t="s">
+      <c r="A92" t="s">
         <v>117</v>
       </c>
       <c r="B92" s="1" t="s">
@@ -3200,7 +3212,7 @@
       </c>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A93" s="10" t="s">
+      <c r="A93" t="s">
         <v>118</v>
       </c>
       <c r="B93" s="1" t="s">
@@ -3224,7 +3236,7 @@
       </c>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A94" s="10" t="s">
+      <c r="A94" t="s">
         <v>119</v>
       </c>
       <c r="B94" s="1" t="s">
@@ -3248,7 +3260,7 @@
       </c>
     </row>
     <row r="95" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A95" s="10" t="s">
+      <c r="A95" t="s">
         <v>120</v>
       </c>
       <c r="B95" s="1" t="s">
@@ -3265,6 +3277,150 @@
         <v>222</v>
       </c>
       <c r="G95" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>246</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C96" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="D96" t="str">
+        <f t="shared" ref="D96:D101" si="4">_xlfn.CONCAT("Engagement - ", C96)</f>
+        <v>Engagement - Philippines</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F96" t="s">
+        <v>238</v>
+      </c>
+      <c r="G96" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>247</v>
+      </c>
+      <c r="B97" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C97" s="2" t="s">
+        <v>241</v>
+      </c>
+      <c r="D97" t="str">
+        <f t="shared" si="4"/>
+        <v>Engagement - Australia</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F97" t="s">
+        <v>238</v>
+      </c>
+      <c r="G97" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>248</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C98" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D98" t="str">
+        <f t="shared" si="4"/>
+        <v>Engagement - North America</v>
+      </c>
+      <c r="E98" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="F98" t="s">
+        <v>238</v>
+      </c>
+      <c r="G98" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>249</v>
+      </c>
+      <c r="B99" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C99" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D99" t="str">
+        <f t="shared" si="4"/>
+        <v>Engagement - North America</v>
+      </c>
+      <c r="E99" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="F99" t="s">
+        <v>238</v>
+      </c>
+      <c r="G99" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>250</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C100" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D100" t="str">
+        <f t="shared" si="4"/>
+        <v>Engagement - North America</v>
+      </c>
+      <c r="E100" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F100" t="s">
+        <v>238</v>
+      </c>
+      <c r="G100" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>251</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C101" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="D101" t="str">
+        <f t="shared" si="4"/>
+        <v>Engagement - North America</v>
+      </c>
+      <c r="E101" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F101" t="s">
+        <v>238</v>
+      </c>
+      <c r="G101" t="s">
         <v>225</v>
       </c>
     </row>

</xml_diff>